<commit_message>
first version of README.md
</commit_message>
<xml_diff>
--- a/runs/bulk_results/validation_12/detail_combined.xlsx
+++ b/runs/bulk_results/validation_12/detail_combined.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Davide\Desktop\POLIMI\Tesi\GitHub_Code\DataAgent-1\runs\bulk_results\validation_12\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB18DBC-2553-4BFA-B778-2D020FC99D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -277,8 +283,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -295,12 +301,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -330,24 +342,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -385,7 +408,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -419,6 +442,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -453,9 +477,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -628,11 +653,40 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BX7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="11" max="11" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.08984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="24.36328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="28.6328125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="28.7265625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="22.6328125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="22.90625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="16.1796875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:76">
+    <row r="1" spans="1:76" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -684,19 +738,19 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
       <c r="W1" s="1" t="s">
@@ -714,19 +768,19 @@
       <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
       <c r="AG1" s="1" t="s">
@@ -862,7 +916,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:76">
+    <row r="2" spans="1:76" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0</v>
       </c>
@@ -900,79 +954,79 @@
         <v>11.24</v>
       </c>
       <c r="M2">
-        <v>8.140000000000001</v>
+        <v>8.14</v>
       </c>
       <c r="N2">
         <v>18.79</v>
       </c>
       <c r="O2">
-        <v>9.946</v>
+        <v>9.9459999999999997</v>
       </c>
       <c r="P2">
-        <v>8.121</v>
+        <v>8.1210000000000004</v>
       </c>
       <c r="Q2">
-        <v>17.492</v>
+        <v>17.492000000000001</v>
       </c>
       <c r="R2">
-        <v>0.0001397466138888</v>
+        <v>1.3974661388880001E-4</v>
       </c>
       <c r="S2">
-        <v>0.0001199288383333</v>
+        <v>1.199288383333E-4</v>
       </c>
       <c r="T2">
         <v>0</v>
       </c>
       <c r="U2">
-        <v>1.981777555553588E-05</v>
+        <v>1.9817775555535879E-5</v>
       </c>
       <c r="V2">
-        <v>4.62167206520886E-05</v>
+        <v>4.6216720652088601E-5</v>
       </c>
       <c r="W2">
-        <v>4.344067833328356E-05</v>
+        <v>4.3440678333283598E-5</v>
       </c>
       <c r="X2">
-        <v>3.727991666661788E-05</v>
+        <v>3.7279916666617883E-5</v>
       </c>
       <c r="Y2">
         <v>0</v>
       </c>
       <c r="Z2">
-        <v>6.160761666665672E-06</v>
+        <v>6.1607616666656722E-6</v>
       </c>
       <c r="AA2">
-        <v>1.436661425702687E-05</v>
+        <v>1.436661425702687E-5</v>
       </c>
       <c r="AB2">
-        <v>0.0001245526972222</v>
+        <v>1.245526972222E-4</v>
       </c>
       <c r="AC2">
-        <v>0.0001069035733333</v>
+        <v>1.069035733333E-4</v>
       </c>
       <c r="AD2">
         <v>0</v>
       </c>
       <c r="AE2">
-        <v>1.76491238888856E-05</v>
+        <v>1.76491238888856E-5</v>
       </c>
       <c r="AF2">
-        <v>4.119181891993651E-05</v>
+        <v>4.1191818919936507E-5</v>
       </c>
       <c r="AG2">
-        <v>0.0009063624363892</v>
+        <v>9.0636243638920002E-4</v>
       </c>
       <c r="AH2">
-        <v>0.0007775746100003</v>
+        <v>7.7757461000030001E-4</v>
       </c>
       <c r="AI2">
         <v>0</v>
       </c>
       <c r="AJ2">
-        <v>0.0001287878263889</v>
+        <v>1.2878782638889999E-4</v>
       </c>
       <c r="AK2">
-        <v>0.0002997503722377</v>
+        <v>2.9975037223770002E-4</v>
       </c>
       <c r="AL2" t="s">
         <v>80</v>
@@ -993,10 +1047,10 @@
         <v>1</v>
       </c>
       <c r="AR2">
-        <v>0.2559</v>
+        <v>0.25590000000000002</v>
       </c>
       <c r="AS2">
-        <v>0.2559</v>
+        <v>0.25590000000000002</v>
       </c>
       <c r="AT2">
         <v>0.755</v>
@@ -1065,7 +1119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:76">
+    <row r="3" spans="1:76" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1112,70 +1166,70 @@
         <v>14.241</v>
       </c>
       <c r="P3">
-        <v>8.461</v>
+        <v>8.4610000000000003</v>
       </c>
       <c r="Q3">
-        <v>14.299</v>
+        <v>14.298999999999999</v>
       </c>
       <c r="R3">
-        <v>0.0001976139527777</v>
+        <v>1.9761395277769999E-4</v>
       </c>
       <c r="S3">
-        <v>0.0001696059583333</v>
+        <v>1.696059583333E-4</v>
       </c>
       <c r="T3">
         <v>0</v>
       </c>
       <c r="U3">
-        <v>2.800799444445753E-05</v>
+        <v>2.8007994444457531E-5</v>
       </c>
       <c r="V3">
-        <v>6.535449123476791E-05</v>
+        <v>6.5354491234767908E-5</v>
       </c>
       <c r="W3">
-        <v>2.598508194444851E-05</v>
+        <v>2.598508194444851E-5</v>
       </c>
       <c r="X3">
-        <v>2.230651500000628E-05</v>
+        <v>2.230651500000628E-5</v>
       </c>
       <c r="Y3">
         <v>0</v>
       </c>
       <c r="Z3">
-        <v>3.678566944442234E-06</v>
+        <v>3.678566944442234E-6</v>
       </c>
       <c r="AA3">
-        <v>8.593734330504123E-06</v>
+        <v>8.5937343305041229E-6</v>
       </c>
       <c r="AB3">
-        <v>7.6227464444542E-05</v>
+        <v>7.6227464444542003E-5</v>
       </c>
       <c r="AC3">
-        <v>6.542664833341405E-05</v>
+        <v>6.5426648333414048E-5</v>
       </c>
       <c r="AD3">
         <v>0</v>
       </c>
       <c r="AE3">
-        <v>1.080081611112796E-05</v>
+        <v>1.080081611112796E-5</v>
       </c>
       <c r="AF3">
-        <v>2.520979458617004E-05</v>
+        <v>2.5209794586170039E-5</v>
       </c>
       <c r="AG3">
-        <v>0.0008822507991664001</v>
+        <v>8.8225079916640005E-4</v>
       </c>
       <c r="AH3">
-        <v>0.0007568249099998</v>
+        <v>7.5682490999980003E-4</v>
       </c>
       <c r="AI3">
         <v>0</v>
       </c>
       <c r="AJ3">
-        <v>0.0001254258891666</v>
+        <v>1.2542588916659999E-4</v>
       </c>
       <c r="AK3">
-        <v>0.0002917762197987</v>
+        <v>2.9177621979870001E-4</v>
       </c>
       <c r="AL3" t="s">
         <v>81</v>
@@ -1196,16 +1250,16 @@
         <v>3</v>
       </c>
       <c r="AR3">
-        <v>0.1312</v>
+        <v>0.13120000000000001</v>
       </c>
       <c r="AS3">
         <v>0.3407</v>
       </c>
       <c r="AT3">
-        <v>0.9599</v>
+        <v>0.95989999999999998</v>
       </c>
       <c r="AU3">
-        <v>0.9599</v>
+        <v>0.95989999999999998</v>
       </c>
       <c r="AV3">
         <v>1500</v>
@@ -1268,7 +1322,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:76">
+    <row r="4" spans="1:76" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>0</v>
       </c>
@@ -1306,13 +1360,13 @@
         <v>3.76</v>
       </c>
       <c r="M4">
-        <v>9.630000000000001</v>
+        <v>9.6300000000000008</v>
       </c>
       <c r="N4">
         <v>15.14</v>
       </c>
       <c r="O4">
-        <v>3.553</v>
+        <v>3.5529999999999999</v>
       </c>
       <c r="P4">
         <v>9.6</v>
@@ -1321,64 +1375,64 @@
         <v>15.06</v>
       </c>
       <c r="R4">
-        <v>5.612912722217516E-05</v>
+        <v>5.6129127222175161E-5</v>
       </c>
       <c r="S4">
-        <v>4.816864499995669E-05</v>
+        <v>4.8168644999956687E-5</v>
       </c>
       <c r="T4">
         <v>0</v>
       </c>
       <c r="U4">
-        <v>7.960482222218465E-06</v>
+        <v>7.9604822222184654E-6</v>
       </c>
       <c r="V4">
-        <v>1.856291269666333E-05</v>
+        <v>1.8562912696663329E-5</v>
       </c>
       <c r="W4">
-        <v>5.645207527787635E-05</v>
+        <v>5.6452075277876347E-5</v>
       </c>
       <c r="X4">
-        <v>4.844142166675738E-05</v>
+        <v>4.8441421666757378E-5</v>
       </c>
       <c r="Y4">
         <v>0</v>
       </c>
       <c r="Z4">
-        <v>8.01065361111897E-06</v>
+        <v>8.0106536111189698E-6</v>
       </c>
       <c r="AA4">
-        <v>1.866971743174871E-05</v>
+        <v>1.8669717431748711E-5</v>
       </c>
       <c r="AB4">
-        <v>8.745290722224834E-05</v>
+        <v>8.7452907222248337E-5</v>
       </c>
       <c r="AC4">
-        <v>7.503488833335723E-05</v>
+        <v>7.5034888333357232E-5</v>
       </c>
       <c r="AD4">
         <v>0</v>
       </c>
       <c r="AE4">
-        <v>1.241801888889111E-05</v>
+        <v>1.2418018888891109E-5</v>
       </c>
       <c r="AF4">
-        <v>2.892225057072753E-05</v>
+        <v>2.8922250570727529E-5</v>
       </c>
       <c r="AG4">
-        <v>0.0006953481172222</v>
+        <v>6.9534811722219998E-4</v>
       </c>
       <c r="AH4">
-        <v>0.0005964618366667</v>
+        <v>5.9646183666669996E-4</v>
       </c>
       <c r="AI4">
         <v>0</v>
       </c>
       <c r="AJ4">
-        <v>9.88862805555578E-05</v>
+        <v>9.8886280555557805E-5</v>
       </c>
       <c r="AK4">
-        <v>0.0002299641386315</v>
+        <v>2.2996413863150001E-4</v>
       </c>
       <c r="AL4" t="s">
         <v>80</v>
@@ -1426,13 +1480,13 @@
         <v>3</v>
       </c>
       <c r="BD4">
-        <v>0.2197</v>
+        <v>0.21970000000000001</v>
       </c>
       <c r="BE4">
-        <v>0.2197</v>
+        <v>0.21970000000000001</v>
       </c>
       <c r="BF4">
-        <v>0.9196</v>
+        <v>0.91959999999999997</v>
       </c>
       <c r="BG4">
         <v>1</v>
@@ -1471,7 +1525,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:76">
+    <row r="5" spans="1:76" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1515,73 +1569,73 @@
         <v>13.23</v>
       </c>
       <c r="O5">
-        <v>2.483</v>
+        <v>2.4830000000000001</v>
       </c>
       <c r="P5">
-        <v>21.719</v>
+        <v>21.719000000000001</v>
       </c>
       <c r="Q5">
         <v>13.119</v>
       </c>
       <c r="R5">
-        <v>3.584802722221461E-05</v>
+        <v>3.5848027222214608E-5</v>
       </c>
       <c r="S5">
-        <v>3.076181999998274E-05</v>
+        <v>3.0761819999982743E-5</v>
       </c>
       <c r="T5">
         <v>0</v>
       </c>
       <c r="U5">
-        <v>5.08620722223188E-06</v>
+        <v>5.0862072222318802E-6</v>
       </c>
       <c r="V5">
-        <v>1.185558786687637E-05</v>
+        <v>1.1855587866876369E-5</v>
       </c>
       <c r="W5">
-        <v>0.0001460478472221</v>
+        <v>1.4604784722209999E-4</v>
       </c>
       <c r="X5">
-        <v>0.0001253248616665</v>
+        <v>1.2532486166649999E-4</v>
       </c>
       <c r="Y5">
         <v>0</v>
       </c>
       <c r="Z5">
-        <v>2.072298555555487E-05</v>
+        <v>2.072298555555487E-5</v>
       </c>
       <c r="AA5">
-        <v>4.830065193760296E-05</v>
+        <v>4.8300651937602957E-5</v>
       </c>
       <c r="AB5">
-        <v>8.172019249995072E-05</v>
+        <v>8.1720192499950723E-5</v>
       </c>
       <c r="AC5">
-        <v>7.013696166662461E-05</v>
+        <v>7.0136961666624609E-5</v>
       </c>
       <c r="AD5">
         <v>0</v>
       </c>
       <c r="AE5">
-        <v>1.158323083332612E-05</v>
+        <v>1.1583230833326119E-5</v>
       </c>
       <c r="AF5">
-        <v>2.70263386231987E-05</v>
+        <v>2.70263386231987E-5</v>
       </c>
       <c r="AG5">
-        <v>0.0008729078624999</v>
+        <v>8.7290786249989997E-4</v>
       </c>
       <c r="AH5">
-        <v>0.0007488275449999</v>
+        <v>7.4882754499990001E-4</v>
       </c>
       <c r="AI5">
         <v>0</v>
       </c>
       <c r="AJ5">
-        <v>0.0001240803175</v>
+        <v>1.240803175E-4</v>
       </c>
       <c r="AK5">
-        <v>0.0002886863424702</v>
+        <v>2.8868634247020001E-4</v>
       </c>
       <c r="AL5" t="s">
         <v>80</v>
@@ -1632,13 +1686,13 @@
         <v>0.12</v>
       </c>
       <c r="BE5">
-        <v>0.6215000000000001</v>
+        <v>0.62150000000000005</v>
       </c>
       <c r="BF5">
-        <v>0.8001</v>
+        <v>0.80010000000000003</v>
       </c>
       <c r="BG5">
-        <v>0.8001</v>
+        <v>0.80010000000000003</v>
       </c>
       <c r="BH5">
         <v>4000</v>
@@ -1674,7 +1728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:76">
+    <row r="6" spans="1:76" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>0</v>
       </c>
@@ -1709,7 +1763,7 @@
         <v>83.47</v>
       </c>
       <c r="L6">
-        <v>2.53</v>
+        <v>2.5299999999999998</v>
       </c>
       <c r="M6">
         <v>6.64</v>
@@ -1718,73 +1772,73 @@
         <v>63.14</v>
       </c>
       <c r="O6">
-        <v>2.309</v>
+        <v>2.3090000000000002</v>
       </c>
       <c r="P6">
-        <v>6.632</v>
+        <v>6.6319999999999997</v>
       </c>
       <c r="Q6">
-        <v>62.721</v>
+        <v>62.720999999999997</v>
       </c>
       <c r="R6">
-        <v>3.093726111114341E-05</v>
+        <v>3.0937261111143407E-5</v>
       </c>
       <c r="S6">
-        <v>2.654955666669896E-05</v>
+        <v>2.6549556666698959E-5</v>
       </c>
       <c r="T6">
         <v>0</v>
       </c>
       <c r="U6">
-        <v>4.387704444444453E-06</v>
+        <v>4.3877044444444534E-6</v>
       </c>
       <c r="V6">
-        <v>1.023150912015513E-05</v>
+        <v>1.023150912015513E-5</v>
       </c>
       <c r="W6">
-        <v>2.355365500002841E-05</v>
+        <v>2.3553655000028411E-5</v>
       </c>
       <c r="X6">
-        <v>2.021244166668718E-05</v>
+        <v>2.021244166668718E-5</v>
       </c>
       <c r="Y6">
         <v>0</v>
       </c>
       <c r="Z6">
-        <v>3.341213333341228E-06</v>
+        <v>3.3412133333412279E-6</v>
       </c>
       <c r="AA6">
-        <v>7.789617674299396E-06</v>
+        <v>7.789617674299396E-6</v>
       </c>
       <c r="AB6">
-        <v>0.0004542250708333</v>
+        <v>4.542250708333E-4</v>
       </c>
       <c r="AC6">
-        <v>0.00038973623</v>
+        <v>3.8973623000000001E-4</v>
       </c>
       <c r="AD6">
         <v>0</v>
       </c>
       <c r="AE6">
-        <v>6.44888408333322E-05</v>
+        <v>6.4488840833332197E-5</v>
       </c>
       <c r="AF6">
-        <v>0.0001502204069758</v>
+        <v>1.5022040697579999E-4</v>
       </c>
       <c r="AG6">
-        <v>0.0016214917963886</v>
+        <v>1.6214917963885999E-3</v>
       </c>
       <c r="AH6">
-        <v>0.0013909170333331</v>
+        <v>1.3909170333330999E-3</v>
       </c>
       <c r="AI6">
         <v>0</v>
       </c>
       <c r="AJ6">
-        <v>0.0002305747630555</v>
+        <v>2.3057476305549999E-4</v>
       </c>
       <c r="AK6">
-        <v>0.000536256523918</v>
+        <v>5.3625652391799995E-4</v>
       </c>
       <c r="AL6" t="s">
         <v>80</v>
@@ -1859,10 +1913,10 @@
         <v>1</v>
       </c>
       <c r="BP6">
-        <v>0.178</v>
+        <v>0.17799999999999999</v>
       </c>
       <c r="BQ6">
-        <v>0.178</v>
+        <v>0.17799999999999999</v>
       </c>
       <c r="BR6">
         <v>0.755</v>
@@ -1877,7 +1931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:76">
+    <row r="7" spans="1:76" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1903,91 +1957,91 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>0.8333</v>
+        <v>0.83330000000000004</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="K7">
-        <v>83.15000000000001</v>
+        <v>83.15</v>
       </c>
       <c r="L7">
         <v>3.98</v>
       </c>
       <c r="M7">
-        <v>8.300000000000001</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="N7">
         <v>63.06</v>
       </c>
       <c r="O7">
-        <v>3.745</v>
+        <v>3.7450000000000001</v>
       </c>
       <c r="P7">
-        <v>8.289999999999999</v>
+        <v>8.2899999999999991</v>
       </c>
       <c r="Q7">
         <v>62.43</v>
       </c>
       <c r="R7">
-        <v>5.942678361121175E-05</v>
+        <v>5.942678361121175E-5</v>
       </c>
       <c r="S7">
-        <v>5.098336666675701E-05</v>
+        <v>5.0983366666757012E-5</v>
       </c>
       <c r="T7">
         <v>0</v>
       </c>
       <c r="U7">
-        <v>8.443416944454738E-06</v>
+        <v>8.4434169444547381E-6</v>
       </c>
       <c r="V7">
-        <v>1.965350702233273E-05</v>
+        <v>1.9653507022332728E-5</v>
       </c>
       <c r="W7">
-        <v>2.46779669445257E-05</v>
+        <v>2.4677966944525701E-5</v>
       </c>
       <c r="X7">
-        <v>2.116732833340696E-05</v>
+        <v>2.116732833340696E-5</v>
       </c>
       <c r="Y7">
         <v>0</v>
       </c>
       <c r="Z7">
-        <v>3.510638611118742E-06</v>
+        <v>3.510638611118742E-6</v>
       </c>
       <c r="AA7">
-        <v>8.161447871959653E-06</v>
+        <v>8.1614478719596528E-6</v>
       </c>
       <c r="AB7">
-        <v>0.0005094706788887</v>
+        <v>5.0947067888869996E-4</v>
       </c>
       <c r="AC7">
-        <v>0.0004371325899999</v>
+        <v>4.3713258999990003E-4</v>
       </c>
       <c r="AD7">
         <v>0</v>
       </c>
       <c r="AE7">
-        <v>7.233808888887426E-05</v>
+        <v>7.2338088888874259E-5</v>
       </c>
       <c r="AF7">
-        <v>0.0001684911239807</v>
+        <v>1.684911239807E-4</v>
       </c>
       <c r="AG7">
-        <v>0.0016151340269443</v>
+        <v>1.6151340269442999E-3</v>
       </c>
       <c r="AH7">
-        <v>0.0013855415666666</v>
+        <v>1.3855415666666E-3</v>
       </c>
       <c r="AI7">
         <v>0</v>
       </c>
       <c r="AJ7">
-        <v>0.0002295924602777</v>
+        <v>2.2959246027769999E-4</v>
       </c>
       <c r="AK7">
-        <v>0.0005341538951228999</v>
+        <v>5.3415389512289995E-4</v>
       </c>
       <c r="AL7" t="s">
         <v>80</v>
@@ -2062,16 +2116,16 @@
         <v>3</v>
       </c>
       <c r="BP7">
-        <v>0.1156</v>
+        <v>0.11559999999999999</v>
       </c>
       <c r="BQ7">
         <v>0.2349</v>
       </c>
       <c r="BR7">
-        <v>0.9599</v>
+        <v>0.95989999999999998</v>
       </c>
       <c r="BS7">
-        <v>0.9599</v>
+        <v>0.95989999999999998</v>
       </c>
       <c r="BT7">
         <v>2000</v>

</xml_diff>